<commit_message>
====== Closing 256 heads transformer
</commit_message>
<xml_diff>
--- a/research/HyperParams.xlsx
+++ b/research/HyperParams.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\Subnet-18-Zeus\research\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E8B2C75-A354-4938-A13C-FA59280F94B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44B98F8C-1D55-4629-ADC4-8C89684CC3A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="11829" xr2:uid="{701B61B4-A6E2-434A-B336-77C79E78CCA1}"/>
   </bookViews>
@@ -111,9 +111,6 @@
     <t>Mode.2</t>
   </si>
   <si>
-    <t>Mode.3</t>
-  </si>
-  <si>
     <t>Mode.4</t>
   </si>
   <si>
@@ -124,6 +121,9 @@
   </si>
   <si>
     <t>Mode.7</t>
+  </si>
+  <si>
+    <t>Mode.3  --- diver</t>
   </si>
 </sst>
 </file>
@@ -535,19 +535,19 @@
         <v>23</v>
       </c>
       <c r="D1" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>27</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>28</v>
       </c>
       <c r="I1" s="3" t="s">
         <v>15</v>
@@ -744,7 +744,7 @@
       <c r="D9" s="7">
         <v>512</v>
       </c>
-      <c r="E9" s="5">
+      <c r="E9" s="7">
         <v>64</v>
       </c>
       <c r="F9" s="5">

</xml_diff>